<commit_message>
feat: initialize disbursement system project with configuration management and logging infrastructure
</commit_message>
<xml_diff>
--- a/disbursement_system/table_main_2569.xlsx
+++ b/disbursement_system/table_main_2569.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="AK26" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4005,7 @@
       </c>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="AK28" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4769,7 +4769,7 @@
       </c>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="AK35" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5293,7 @@
       </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="AK39" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5686,7 @@
       </c>
       <c r="AK40" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5817,7 @@
       </c>
       <c r="AK41" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="AK42" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="AK43" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6210,7 @@
       </c>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6341,7 +6341,7 @@
       </c>
       <c r="AK45" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="AK46" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="AK47" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="AK48" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -6986,7 +6986,7 @@
       </c>
       <c r="AK50" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7117,7 +7117,7 @@
       </c>
       <c r="AK51" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="AK52" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7379,7 @@
       </c>
       <c r="AK53" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="AK54" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7641,7 +7641,7 @@
       </c>
       <c r="AK55" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AK56" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -7903,7 +7903,7 @@
       </c>
       <c r="AK57" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8034,7 +8034,7 @@
       </c>
       <c r="AK58" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="AK59" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="AK60" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8427,7 +8427,7 @@
       </c>
       <c r="AK61" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="AK62" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="AK63" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8820,7 +8820,7 @@
       </c>
       <c r="AK64" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="AK65" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="AK66" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9213,7 +9213,7 @@
       </c>
       <c r="AK67" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="AK68" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9475,7 +9475,7 @@
       </c>
       <c r="AK69" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9606,7 +9606,7 @@
       </c>
       <c r="AK70" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9737,7 +9737,7 @@
       </c>
       <c r="AK71" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -9868,7 +9868,7 @@
       </c>
       <c r="AK72" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="AK73" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10134,7 @@
       </c>
       <c r="AK74" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10269,7 +10269,7 @@
       </c>
       <c r="AK75" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AK76" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10535,7 @@
       </c>
       <c r="AK77" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10668,7 +10668,7 @@
       </c>
       <c r="AK78" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
       </c>
       <c r="AK79" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="AK80" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11069,7 +11069,7 @@
       </c>
       <c r="AK81" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="AK82" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11335,7 +11335,7 @@
       </c>
       <c r="AK83" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11468,7 +11468,7 @@
       </c>
       <c r="AK84" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11601,7 +11601,7 @@
       </c>
       <c r="AK85" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="AK86" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -11867,7 +11867,7 @@
       </c>
       <c r="AK87" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12111,7 +12111,7 @@
       </c>
       <c r="AK89" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12244,7 +12244,7 @@
       </c>
       <c r="AK90" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12377,7 +12377,7 @@
       </c>
       <c r="AK91" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12510,7 +12510,7 @@
       </c>
       <c r="AK92" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12643,7 +12643,7 @@
       </c>
       <c r="AK93" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12776,7 +12776,7 @@
       </c>
       <c r="AK94" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -12909,7 +12909,7 @@
       </c>
       <c r="AK95" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13044,7 +13044,7 @@
       </c>
       <c r="AK96" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="AK97" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="AK98" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13443,7 +13443,7 @@
       </c>
       <c r="AK99" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13576,7 +13576,7 @@
       </c>
       <c r="AK100" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13709,7 +13709,7 @@
       </c>
       <c r="AK101" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13842,7 +13842,7 @@
       </c>
       <c r="AK102" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -13975,7 +13975,7 @@
       </c>
       <c r="AK103" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14108,7 +14108,7 @@
       </c>
       <c r="AK104" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14241,7 +14241,7 @@
       </c>
       <c r="AK105" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14374,7 +14374,7 @@
       </c>
       <c r="AK106" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14507,7 +14507,7 @@
       </c>
       <c r="AK107" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14640,7 +14640,7 @@
       </c>
       <c r="AK108" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14773,7 +14773,7 @@
       </c>
       <c r="AK109" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -14906,7 +14906,7 @@
       </c>
       <c r="AK110" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15039,7 +15039,7 @@
       </c>
       <c r="AK111" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15172,7 +15172,7 @@
       </c>
       <c r="AK112" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="AK113" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15438,7 +15438,7 @@
       </c>
       <c r="AK114" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15571,7 +15571,7 @@
       </c>
       <c r="AK115" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15704,7 +15704,7 @@
       </c>
       <c r="AK116" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15837,7 +15837,7 @@
       </c>
       <c r="AK117" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -15960,7 +15960,7 @@
       </c>
       <c r="AK118" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16093,7 +16093,7 @@
       </c>
       <c r="AK119" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16226,7 +16226,7 @@
       </c>
       <c r="AK120" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16359,7 +16359,7 @@
       </c>
       <c r="AK121" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16492,7 +16492,7 @@
       </c>
       <c r="AK122" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16625,7 +16625,7 @@
       </c>
       <c r="AK123" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16758,7 +16758,7 @@
       </c>
       <c r="AK124" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -16891,7 +16891,7 @@
       </c>
       <c r="AK125" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17024,7 +17024,7 @@
       </c>
       <c r="AK126" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17157,7 +17157,7 @@
       </c>
       <c r="AK127" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17292,7 +17292,7 @@
       </c>
       <c r="AK128" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17425,7 +17425,7 @@
       </c>
       <c r="AK129" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17558,7 +17558,7 @@
       </c>
       <c r="AK130" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17691,7 +17691,7 @@
       </c>
       <c r="AK131" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17824,7 +17824,7 @@
       </c>
       <c r="AK132" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -17957,7 +17957,7 @@
       </c>
       <c r="AK133" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18080,7 +18080,7 @@
       </c>
       <c r="AK134" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18213,7 +18213,7 @@
       </c>
       <c r="AK135" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18346,7 +18346,7 @@
       </c>
       <c r="AK136" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18479,7 +18479,7 @@
       </c>
       <c r="AK137" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18612,7 +18612,7 @@
       </c>
       <c r="AK138" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="AK139" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -18878,7 +18878,7 @@
       </c>
       <c r="AK140" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19011,7 +19011,7 @@
       </c>
       <c r="AK141" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19144,7 +19144,7 @@
       </c>
       <c r="AK142" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19277,7 +19277,7 @@
       </c>
       <c r="AK143" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19408,7 +19408,7 @@
       </c>
       <c r="AK144" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19539,7 +19539,7 @@
       </c>
       <c r="AK145" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19670,7 +19670,7 @@
       </c>
       <c r="AK146" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="AK147" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -19932,7 +19932,7 @@
       </c>
       <c r="AK148" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20063,7 +20063,7 @@
       </c>
       <c r="AK149" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20194,7 +20194,7 @@
       </c>
       <c r="AK150" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="AK151" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20456,7 +20456,7 @@
       </c>
       <c r="AK152" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20587,7 +20587,7 @@
       </c>
       <c r="AK153" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20718,7 +20718,7 @@
       </c>
       <c r="AK154" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20849,7 +20849,7 @@
       </c>
       <c r="AK155" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -20980,7 +20980,7 @@
       </c>
       <c r="AK156" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21111,7 +21111,7 @@
       </c>
       <c r="AK157" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21242,7 +21242,7 @@
       </c>
       <c r="AK158" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21373,7 +21373,7 @@
       </c>
       <c r="AK159" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21504,7 +21504,7 @@
       </c>
       <c r="AK160" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21635,7 +21635,7 @@
       </c>
       <c r="AK161" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21766,7 +21766,7 @@
       </c>
       <c r="AK162" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -21897,7 +21897,7 @@
       </c>
       <c r="AK163" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22028,7 +22028,7 @@
       </c>
       <c r="AK164" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22159,7 +22159,7 @@
       </c>
       <c r="AK165" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22290,7 +22290,7 @@
       </c>
       <c r="AK166" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22421,7 +22421,7 @@
       </c>
       <c r="AK167" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22552,7 +22552,7 @@
       </c>
       <c r="AK168" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22683,7 +22683,7 @@
       </c>
       <c r="AK169" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22814,7 +22814,7 @@
       </c>
       <c r="AK170" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -22945,7 +22945,7 @@
       </c>
       <c r="AK171" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23076,7 +23076,7 @@
       </c>
       <c r="AK172" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23207,7 +23207,7 @@
       </c>
       <c r="AK173" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23338,7 +23338,7 @@
       </c>
       <c r="AK174" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23469,7 +23469,7 @@
       </c>
       <c r="AK175" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23600,7 +23600,7 @@
       </c>
       <c r="AK176" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23731,7 +23731,7 @@
       </c>
       <c r="AK177" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23862,7 +23862,7 @@
       </c>
       <c r="AK178" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -23993,7 +23993,7 @@
       </c>
       <c r="AK179" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24124,7 +24124,7 @@
       </c>
       <c r="AK180" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24259,7 +24259,7 @@
       </c>
       <c r="AK181" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24396,7 +24396,7 @@
       </c>
       <c r="AK182" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24533,7 +24533,7 @@
       </c>
       <c r="AK183" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24668,7 +24668,7 @@
       </c>
       <c r="AK184" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24803,7 +24803,7 @@
       </c>
       <c r="AK185" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -24938,7 +24938,7 @@
       </c>
       <c r="AK186" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25073,7 +25073,7 @@
       </c>
       <c r="AK187" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25208,7 +25208,7 @@
       </c>
       <c r="AK188" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25343,7 +25343,7 @@
       </c>
       <c r="AK189" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25478,7 +25478,7 @@
       </c>
       <c r="AK190" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25613,7 +25613,7 @@
       </c>
       <c r="AK191" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25748,7 +25748,7 @@
       </c>
       <c r="AK192" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -25883,7 +25883,7 @@
       </c>
       <c r="AK193" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26018,7 +26018,7 @@
       </c>
       <c r="AK194" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26153,7 +26153,7 @@
       </c>
       <c r="AK195" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26288,7 +26288,7 @@
       </c>
       <c r="AK196" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26423,7 +26423,7 @@
       </c>
       <c r="AK197" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26558,7 +26558,7 @@
       </c>
       <c r="AK198" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26695,7 +26695,7 @@
       </c>
       <c r="AK199" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26830,7 +26830,7 @@
       </c>
       <c r="AK200" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -26965,7 +26965,7 @@
       </c>
       <c r="AK201" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27100,7 +27100,7 @@
       </c>
       <c r="AK202" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27235,7 +27235,7 @@
       </c>
       <c r="AK203" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27370,7 +27370,7 @@
       </c>
       <c r="AK204" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27505,7 +27505,7 @@
       </c>
       <c r="AK205" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27640,7 +27640,7 @@
       </c>
       <c r="AK206" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27775,7 +27775,7 @@
       </c>
       <c r="AK207" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -27910,7 +27910,7 @@
       </c>
       <c r="AK208" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28045,7 +28045,7 @@
       </c>
       <c r="AK209" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28180,7 +28180,7 @@
       </c>
       <c r="AK210" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28315,7 +28315,7 @@
       </c>
       <c r="AK211" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28450,7 +28450,7 @@
       </c>
       <c r="AK212" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28577,7 +28577,7 @@
       </c>
       <c r="AK213" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28712,7 +28712,7 @@
       </c>
       <c r="AK214" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28847,7 +28847,7 @@
       </c>
       <c r="AK215" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -28982,7 +28982,7 @@
       </c>
       <c r="AK216" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29117,7 +29117,7 @@
       </c>
       <c r="AK217" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29252,7 +29252,7 @@
       </c>
       <c r="AK218" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29389,7 +29389,7 @@
       </c>
       <c r="AK219" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29526,7 +29526,7 @@
       </c>
       <c r="AK220" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29661,7 +29661,7 @@
       </c>
       <c r="AK221" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29796,7 +29796,7 @@
       </c>
       <c r="AK222" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -29931,7 +29931,7 @@
       </c>
       <c r="AK223" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30066,7 +30066,7 @@
       </c>
       <c r="AK224" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30201,7 +30201,7 @@
       </c>
       <c r="AK225" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30336,7 +30336,7 @@
       </c>
       <c r="AK226" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30471,7 +30471,7 @@
       </c>
       <c r="AK227" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30606,7 +30606,7 @@
       </c>
       <c r="AK228" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30741,7 +30741,7 @@
       </c>
       <c r="AK229" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -30876,7 +30876,7 @@
       </c>
       <c r="AK230" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31011,7 +31011,7 @@
       </c>
       <c r="AK231" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31146,7 +31146,7 @@
       </c>
       <c r="AK232" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31281,7 +31281,7 @@
       </c>
       <c r="AK233" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31416,7 +31416,7 @@
       </c>
       <c r="AK234" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31551,7 +31551,7 @@
       </c>
       <c r="AK235" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31686,7 +31686,7 @@
       </c>
       <c r="AK236" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31821,7 +31821,7 @@
       </c>
       <c r="AK237" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -31956,7 +31956,7 @@
       </c>
       <c r="AK238" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32091,7 +32091,7 @@
       </c>
       <c r="AK239" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32226,7 +32226,7 @@
       </c>
       <c r="AK240" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32361,7 +32361,7 @@
       </c>
       <c r="AK241" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32496,7 +32496,7 @@
       </c>
       <c r="AK242" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32631,7 +32631,7 @@
       </c>
       <c r="AK243" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32766,7 +32766,7 @@
       </c>
       <c r="AK244" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -32901,7 +32901,7 @@
       </c>
       <c r="AK245" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33036,7 +33036,7 @@
       </c>
       <c r="AK246" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33171,7 +33171,7 @@
       </c>
       <c r="AK247" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33306,7 +33306,7 @@
       </c>
       <c r="AK248" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33441,7 +33441,7 @@
       </c>
       <c r="AK249" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33576,7 +33576,7 @@
       </c>
       <c r="AK250" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33711,7 +33711,7 @@
       </c>
       <c r="AK251" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33846,7 +33846,7 @@
       </c>
       <c r="AK252" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -33981,7 +33981,7 @@
       </c>
       <c r="AK253" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34116,7 +34116,7 @@
       </c>
       <c r="AK254" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34251,7 +34251,7 @@
       </c>
       <c r="AK255" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34386,7 +34386,7 @@
       </c>
       <c r="AK256" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34521,7 +34521,7 @@
       </c>
       <c r="AK257" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34656,7 +34656,7 @@
       </c>
       <c r="AK258" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34791,7 +34791,7 @@
       </c>
       <c r="AK259" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -34926,7 +34926,7 @@
       </c>
       <c r="AK260" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35061,7 +35061,7 @@
       </c>
       <c r="AK261" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35196,7 +35196,7 @@
       </c>
       <c r="AK262" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35331,7 +35331,7 @@
       </c>
       <c r="AK263" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35466,7 +35466,7 @@
       </c>
       <c r="AK264" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35591,7 +35591,7 @@
       </c>
       <c r="AK265" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35726,7 +35726,7 @@
       </c>
       <c r="AK266" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35861,7 +35861,7 @@
       </c>
       <c r="AK267" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -35996,7 +35996,7 @@
       </c>
       <c r="AK268" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36131,7 +36131,7 @@
       </c>
       <c r="AK269" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36266,7 +36266,7 @@
       </c>
       <c r="AK270" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36401,7 +36401,7 @@
       </c>
       <c r="AK271" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36536,7 +36536,7 @@
       </c>
       <c r="AK272" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36671,7 +36671,7 @@
       </c>
       <c r="AK273" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36806,7 +36806,7 @@
       </c>
       <c r="AK274" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -36941,7 +36941,7 @@
       </c>
       <c r="AK275" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37076,7 +37076,7 @@
       </c>
       <c r="AK276" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37211,7 +37211,7 @@
       </c>
       <c r="AK277" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37346,7 +37346,7 @@
       </c>
       <c r="AK278" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37481,7 +37481,7 @@
       </c>
       <c r="AK279" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37616,7 +37616,7 @@
       </c>
       <c r="AK280" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37751,7 +37751,7 @@
       </c>
       <c r="AK281" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -37886,7 +37886,7 @@
       </c>
       <c r="AK282" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38021,7 +38021,7 @@
       </c>
       <c r="AK283" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38156,7 +38156,7 @@
       </c>
       <c r="AK284" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
       </c>
       <c r="AK285" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38426,7 +38426,7 @@
       </c>
       <c r="AK286" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38561,7 +38561,7 @@
       </c>
       <c r="AK287" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38696,7 +38696,7 @@
       </c>
       <c r="AK288" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38831,7 +38831,7 @@
       </c>
       <c r="AK289" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -38966,7 +38966,7 @@
       </c>
       <c r="AK290" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39101,7 +39101,7 @@
       </c>
       <c r="AK291" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39236,7 +39236,7 @@
       </c>
       <c r="AK292" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39371,7 +39371,7 @@
       </c>
       <c r="AK293" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39506,7 +39506,7 @@
       </c>
       <c r="AK294" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39641,7 +39641,7 @@
       </c>
       <c r="AK295" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39776,7 +39776,7 @@
       </c>
       <c r="AK296" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -39911,7 +39911,7 @@
       </c>
       <c r="AK297" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40046,7 +40046,7 @@
       </c>
       <c r="AK298" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40177,7 +40177,7 @@
       </c>
       <c r="AK299" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40312,7 +40312,7 @@
       </c>
       <c r="AK300" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40447,7 +40447,7 @@
       </c>
       <c r="AK301" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40582,7 +40582,7 @@
       </c>
       <c r="AK302" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40717,7 +40717,7 @@
       </c>
       <c r="AK303" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40852,7 +40852,7 @@
       </c>
       <c r="AK304" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -40987,7 +40987,7 @@
       </c>
       <c r="AK305" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41122,7 +41122,7 @@
       </c>
       <c r="AK306" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41255,7 +41255,7 @@
       </c>
       <c r="AK307" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41390,7 +41390,7 @@
       </c>
       <c r="AK308" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41525,7 +41525,7 @@
       </c>
       <c r="AK309" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41660,7 +41660,7 @@
       </c>
       <c r="AK310" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41795,7 +41795,7 @@
       </c>
       <c r="AK311" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -41932,7 +41932,7 @@
       </c>
       <c r="AK312" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42067,7 +42067,7 @@
       </c>
       <c r="AK313" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42202,7 +42202,7 @@
       </c>
       <c r="AK314" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42337,7 +42337,7 @@
       </c>
       <c r="AK315" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42472,7 +42472,7 @@
       </c>
       <c r="AK316" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42607,7 +42607,7 @@
       </c>
       <c r="AK317" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42742,7 +42742,7 @@
       </c>
       <c r="AK318" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -42877,7 +42877,7 @@
       </c>
       <c r="AK319" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43012,7 +43012,7 @@
       </c>
       <c r="AK320" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43147,7 +43147,7 @@
       </c>
       <c r="AK321" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43282,7 +43282,7 @@
       </c>
       <c r="AK322" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43417,7 +43417,7 @@
       </c>
       <c r="AK323" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43552,7 +43552,7 @@
       </c>
       <c r="AK324" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43687,7 +43687,7 @@
       </c>
       <c r="AK325" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43822,7 +43822,7 @@
       </c>
       <c r="AK326" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -43957,7 +43957,7 @@
       </c>
       <c r="AK327" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44092,7 +44092,7 @@
       </c>
       <c r="AK328" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44227,7 +44227,7 @@
       </c>
       <c r="AK329" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44362,7 +44362,7 @@
       </c>
       <c r="AK330" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44497,7 +44497,7 @@
       </c>
       <c r="AK331" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44632,7 +44632,7 @@
       </c>
       <c r="AK332" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44767,7 +44767,7 @@
       </c>
       <c r="AK333" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -44902,7 +44902,7 @@
       </c>
       <c r="AK334" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45033,7 +45033,7 @@
       </c>
       <c r="AK335" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45168,7 +45168,7 @@
       </c>
       <c r="AK336" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45303,7 +45303,7 @@
       </c>
       <c r="AK337" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45438,7 +45438,7 @@
       </c>
       <c r="AK338" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45573,7 +45573,7 @@
       </c>
       <c r="AK339" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45710,7 +45710,7 @@
       </c>
       <c r="AK340" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45845,7 +45845,7 @@
       </c>
       <c r="AK341" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -45980,7 +45980,7 @@
       </c>
       <c r="AK342" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46115,7 +46115,7 @@
       </c>
       <c r="AK343" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46250,7 +46250,7 @@
       </c>
       <c r="AK344" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46385,7 +46385,7 @@
       </c>
       <c r="AK345" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46520,7 +46520,7 @@
       </c>
       <c r="AK346" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46655,7 +46655,7 @@
       </c>
       <c r="AK347" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46790,7 +46790,7 @@
       </c>
       <c r="AK348" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -46915,7 +46915,7 @@
       </c>
       <c r="AK349" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47050,7 +47050,7 @@
       </c>
       <c r="AK350" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47185,7 +47185,7 @@
       </c>
       <c r="AK351" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47316,7 +47316,7 @@
       </c>
       <c r="AK352" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47447,7 +47447,7 @@
       </c>
       <c r="AK353" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47578,7 +47578,7 @@
       </c>
       <c r="AK354" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47709,7 +47709,7 @@
       </c>
       <c r="AK355" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47840,7 +47840,7 @@
       </c>
       <c r="AK356" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -47971,7 +47971,7 @@
       </c>
       <c r="AK357" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48102,7 +48102,7 @@
       </c>
       <c r="AK358" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48233,7 +48233,7 @@
       </c>
       <c r="AK359" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48364,7 +48364,7 @@
       </c>
       <c r="AK360" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48495,7 +48495,7 @@
       </c>
       <c r="AK361" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48626,7 +48626,7 @@
       </c>
       <c r="AK362" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48757,7 +48757,7 @@
       </c>
       <c r="AK363" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -48888,7 +48888,7 @@
       </c>
       <c r="AK364" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49019,7 +49019,7 @@
       </c>
       <c r="AK365" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49150,7 +49150,7 @@
       </c>
       <c r="AK366" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49281,7 +49281,7 @@
       </c>
       <c r="AK367" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49412,7 +49412,7 @@
       </c>
       <c r="AK368" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49543,7 +49543,7 @@
       </c>
       <c r="AK369" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49674,7 +49674,7 @@
       </c>
       <c r="AK370" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49805,7 +49805,7 @@
       </c>
       <c r="AK371" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -49936,7 +49936,7 @@
       </c>
       <c r="AK372" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50067,7 +50067,7 @@
       </c>
       <c r="AK373" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50198,7 +50198,7 @@
       </c>
       <c r="AK374" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50329,7 +50329,7 @@
       </c>
       <c r="AK375" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50460,7 +50460,7 @@
       </c>
       <c r="AK376" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50591,7 +50591,7 @@
       </c>
       <c r="AK377" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50722,7 +50722,7 @@
       </c>
       <c r="AK378" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50853,7 +50853,7 @@
       </c>
       <c r="AK379" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -50984,7 +50984,7 @@
       </c>
       <c r="AK380" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51115,7 +51115,7 @@
       </c>
       <c r="AK381" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51246,7 +51246,7 @@
       </c>
       <c r="AK382" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51377,7 +51377,7 @@
       </c>
       <c r="AK383" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51508,7 +51508,7 @@
       </c>
       <c r="AK384" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51639,7 +51639,7 @@
       </c>
       <c r="AK385" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51770,7 +51770,7 @@
       </c>
       <c r="AK386" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -51901,7 +51901,7 @@
       </c>
       <c r="AK387" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52032,7 +52032,7 @@
       </c>
       <c r="AK388" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52163,7 +52163,7 @@
       </c>
       <c r="AK389" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52294,7 +52294,7 @@
       </c>
       <c r="AK390" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52425,7 +52425,7 @@
       </c>
       <c r="AK391" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52556,7 +52556,7 @@
       </c>
       <c r="AK392" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52687,7 +52687,7 @@
       </c>
       <c r="AK393" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52818,7 +52818,7 @@
       </c>
       <c r="AK394" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -52949,7 +52949,7 @@
       </c>
       <c r="AK395" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53080,7 +53080,7 @@
       </c>
       <c r="AK396" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53211,7 +53211,7 @@
       </c>
       <c r="AK397" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53342,7 +53342,7 @@
       </c>
       <c r="AK398" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53473,7 +53473,7 @@
       </c>
       <c r="AK399" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53604,7 +53604,7 @@
       </c>
       <c r="AK400" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53735,7 +53735,7 @@
       </c>
       <c r="AK401" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53866,7 +53866,7 @@
       </c>
       <c r="AK402" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -53997,7 +53997,7 @@
       </c>
       <c r="AK403" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54128,7 +54128,7 @@
       </c>
       <c r="AK404" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54259,7 +54259,7 @@
       </c>
       <c r="AK405" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54390,7 +54390,7 @@
       </c>
       <c r="AK406" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54521,7 +54521,7 @@
       </c>
       <c r="AK407" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54652,7 +54652,7 @@
       </c>
       <c r="AK408" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54783,7 +54783,7 @@
       </c>
       <c r="AK409" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -54914,7 +54914,7 @@
       </c>
       <c r="AK410" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -55045,7 +55045,7 @@
       </c>
       <c r="AK411" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -55176,7 +55176,7 @@
       </c>
       <c r="AK412" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -55307,7 +55307,7 @@
       </c>
       <c r="AK413" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>
@@ -55438,7 +55438,7 @@
       </c>
       <c r="AK414" t="inlineStr">
         <is>
-          <t>07/05/2026 15:33</t>
+          <t>07/05/2026 16:24</t>
         </is>
       </c>
     </row>

</xml_diff>